<commit_message>
qol: apply verified +50 lightning resistance bound to Celebrities party
apply verified +50 lightning resistance bound to Celebrities party skill

- Update PartySkillBounds in qol_rules.xlsx (Effect 373 capped at 50 in
x86 code 0x4f92f4) - Regenerate qol_party_skill_text.xlsx (all 20 party
skills now carry exact bounds) - Update test assertion in
test_qol_items_and_install.py - Rebuild and install into
DungeonTravelers2-2_EN/Data/ENG/Parameter/ - All 196 tests passing
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/qol_party_skill_text.xlsx
+++ b/mod_project/data_tables/qol_party_skill_text.xlsx
@@ -1030,17 +1030,21 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Lightning resistance increased.</t>
+          <t>Lightning resistance increased (up to +50).</t>
         </is>
       </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="n">
         <v>373</v>
       </c>
-      <c r="H15" t="inlineStr"/>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>+50</t>
+        </is>
+      </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>The wiki gives no figure</t>
+          <t>exe-verified (0x4f92f4)</t>
         </is>
       </c>
     </row>

</xml_diff>